<commit_message>
button + Speichern.php update
</commit_message>
<xml_diff>
--- a/Content/Guntt_Chart_iii.xlsx
+++ b/Content/Guntt_Chart_iii.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr showObjects="none" filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="731" documentId="13_ncr:1_{F4B7A9DE-D724-4D76-9215-FF6B037D20B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FD7CEC00-3801-47BE-8450-D989F9E56F80}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{80C20573-E1D6-4A5E-BEF9-BD9B0AA8636D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9032B307-AB7D-4148-BD4C-3D4101FE65BD}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Projektplan" sheetId="11" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="256" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="250" uniqueCount="187">
   <si>
     <t>Erstellen Sie auf diesem Arbeitsblatt einen Projektplan.
 Geben Sie den Titel dieses Projekts in Zelle B1 ein. 
@@ -187,15 +187,6 @@
   </si>
   <si>
     <t>Highlight-Formular</t>
-  </si>
-  <si>
-    <t>Admin-Login</t>
-  </si>
-  <si>
-    <t>Pending-Liste</t>
-  </si>
-  <si>
-    <t>Freigeben-Ablehnen</t>
   </si>
   <si>
     <t>Admin-UI Layout</t>
@@ -1834,13 +1825,6 @@
     <dxf>
       <fill>
         <patternFill>
-          <bgColor rgb="FFC00000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
           <bgColor theme="7"/>
         </patternFill>
       </fill>
@@ -1860,6 +1844,13 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC00000"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
       <border>
@@ -2384,7 +2375,7 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:BL55"/>
+  <dimension ref="A1:BL52"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.7109375" style="45" customWidth="1"/>
@@ -2431,7 +2422,7 @@
       <c r="D3" s="94"/>
       <c r="E3" s="98">
         <f ca="1">TODAY()</f>
-        <v>46300</v>
+        <v>46303</v>
       </c>
       <c r="F3" s="98"/>
     </row>
@@ -2858,7 +2849,7 @@
       <c r="F8" s="70"/>
       <c r="G8" s="14"/>
       <c r="H8" s="14" t="str">
-        <f t="shared" ref="H8:H52" si="0">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f t="shared" ref="H8:H49" si="0">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="I8" s="31"/>
@@ -2929,7 +2920,7 @@
         <v>20</v>
       </c>
       <c r="D9" s="17">
-        <v>0.5</v>
+        <v>0.8</v>
       </c>
       <c r="E9" s="81">
         <v>46296.041666666664</v>
@@ -3010,7 +3001,7 @@
         <v>20</v>
       </c>
       <c r="D10" s="17">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E10" s="81">
         <v>46296.125</v>
@@ -3089,7 +3080,7 @@
         <v>20</v>
       </c>
       <c r="D11" s="17">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E11" s="81">
         <v>46296.208333333336</v>
@@ -3167,7 +3158,9 @@
       <c r="C12" s="53" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="17"/>
+      <c r="D12" s="17">
+        <v>1</v>
+      </c>
       <c r="E12" s="81">
         <v>46296.041666666664</v>
       </c>
@@ -3244,7 +3237,9 @@
       <c r="C13" s="59" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="26"/>
+      <c r="D13" s="26">
+        <v>1</v>
+      </c>
       <c r="E13" s="86">
         <v>46301.125</v>
       </c>
@@ -3321,7 +3316,7 @@
         <v>20</v>
       </c>
       <c r="D14" s="17">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="81">
         <v>46302.125</v>
@@ -3470,7 +3465,9 @@
       <c r="C16" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="D16" s="20"/>
+      <c r="D16" s="20">
+        <v>0.3</v>
+      </c>
       <c r="E16" s="84">
         <v>46300.208333333336</v>
       </c>
@@ -3547,7 +3544,9 @@
       <c r="C17" s="55" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="20"/>
+      <c r="D17" s="20">
+        <v>0.2</v>
+      </c>
       <c r="E17" s="84">
         <v>46300.041666666664</v>
       </c>
@@ -3852,7 +3851,7 @@
         <v>36</v>
       </c>
       <c r="C21" s="55" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D21" s="20"/>
       <c r="E21" s="84">
@@ -3926,14 +3925,14 @@
         <v>37</v>
       </c>
       <c r="C22" s="55" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D22" s="20"/>
       <c r="E22" s="84">
         <v>46301.166666666664</v>
       </c>
       <c r="F22" s="84">
-        <v>46301.25</v>
+        <v>46301.291666666664</v>
       </c>
       <c r="G22" s="14"/>
       <c r="H22" s="14"/>
@@ -4000,17 +3999,20 @@
         <v>38</v>
       </c>
       <c r="C23" s="55" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D23" s="20"/>
       <c r="E23" s="84">
-        <v>46301.25</v>
+        <v>46301.041666666664</v>
       </c>
       <c r="F23" s="84">
-        <v>46301.291666666664</v>
+        <v>46301.125</v>
       </c>
       <c r="G23" s="14"/>
-      <c r="H23" s="14"/>
+      <c r="H23" s="14">
+        <f t="shared" si="0"/>
+        <v>1.0833333333357587</v>
+      </c>
       <c r="I23" s="31"/>
       <c r="J23" s="31"/>
       <c r="K23" s="31"/>
@@ -4027,7 +4029,7 @@
       <c r="V23" s="31"/>
       <c r="W23" s="31"/>
       <c r="X23" s="31"/>
-      <c r="Y23" s="32"/>
+      <c r="Y23" s="31"/>
       <c r="Z23" s="31"/>
       <c r="AA23" s="31"/>
       <c r="AB23" s="31"/>
@@ -4070,21 +4072,18 @@
     </row>
     <row r="24" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="45"/>
-      <c r="B24" s="62" t="s">
+      <c r="B24" s="21" t="s">
         <v>39</v>
       </c>
-      <c r="C24" s="55" t="s">
-        <v>32</v>
-      </c>
-      <c r="D24" s="20"/>
-      <c r="E24" s="84">
-        <v>46301.041666666664</v>
-      </c>
-      <c r="F24" s="84">
-        <v>46301.166666666664</v>
-      </c>
+      <c r="C24" s="56"/>
+      <c r="D24" s="22"/>
+      <c r="E24" s="73"/>
+      <c r="F24" s="74"/>
       <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
+      <c r="H24" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="I24" s="31"/>
       <c r="J24" s="31"/>
       <c r="K24" s="31"/>
@@ -4101,7 +4100,7 @@
       <c r="V24" s="31"/>
       <c r="W24" s="31"/>
       <c r="X24" s="31"/>
-      <c r="Y24" s="32"/>
+      <c r="Y24" s="31"/>
       <c r="Z24" s="31"/>
       <c r="AA24" s="31"/>
       <c r="AB24" s="31"/>
@@ -4144,21 +4143,24 @@
     </row>
     <row r="25" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="45"/>
-      <c r="B25" s="62" t="s">
+      <c r="B25" s="63" t="s">
         <v>40</v>
       </c>
-      <c r="C25" s="55" t="s">
+      <c r="C25" s="57" t="s">
         <v>32</v>
       </c>
-      <c r="D25" s="20"/>
-      <c r="E25" s="84">
-        <v>46301.166666666664</v>
-      </c>
-      <c r="F25" s="84">
-        <v>46301.291666666664</v>
+      <c r="D25" s="23"/>
+      <c r="E25" s="85">
+        <v>46302.041666666664</v>
+      </c>
+      <c r="F25" s="85">
+        <v>46302.166666666664</v>
       </c>
       <c r="G25" s="14"/>
-      <c r="H25" s="14"/>
+      <c r="H25" s="14">
+        <f t="shared" si="0"/>
+        <v>1.125</v>
+      </c>
       <c r="I25" s="31"/>
       <c r="J25" s="31"/>
       <c r="K25" s="31"/>
@@ -4175,7 +4177,7 @@
       <c r="V25" s="31"/>
       <c r="W25" s="31"/>
       <c r="X25" s="31"/>
-      <c r="Y25" s="32"/>
+      <c r="Y25" s="31"/>
       <c r="Z25" s="31"/>
       <c r="AA25" s="31"/>
       <c r="AB25" s="31"/>
@@ -4220,18 +4222,18 @@
       <c r="A26" s="45" t="s">
         <v>34</v>
       </c>
-      <c r="B26" s="62" t="s">
+      <c r="B26" s="63" t="s">
         <v>41</v>
       </c>
-      <c r="C26" s="55" t="s">
-        <v>32</v>
-      </c>
-      <c r="D26" s="20"/>
-      <c r="E26" s="84">
-        <v>46301.041666666664</v>
-      </c>
-      <c r="F26" s="84">
-        <v>46301.125</v>
+      <c r="C26" s="57" t="s">
+        <v>20</v>
+      </c>
+      <c r="D26" s="23"/>
+      <c r="E26" s="85">
+        <v>46302.166666666664</v>
+      </c>
+      <c r="F26" s="85">
+        <v>46302.25</v>
       </c>
       <c r="G26" s="14"/>
       <c r="H26" s="14">
@@ -4297,17 +4299,23 @@
     </row>
     <row r="27" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="45"/>
-      <c r="B27" s="21" t="s">
+      <c r="B27" s="63" t="s">
         <v>42</v>
       </c>
-      <c r="C27" s="56"/>
-      <c r="D27" s="22"/>
-      <c r="E27" s="73"/>
-      <c r="F27" s="74"/>
+      <c r="C27" s="57" t="s">
+        <v>20</v>
+      </c>
+      <c r="D27" s="23"/>
+      <c r="E27" s="85">
+        <v>46302.25</v>
+      </c>
+      <c r="F27" s="85">
+        <v>46302.291666666664</v>
+      </c>
       <c r="G27" s="14"/>
-      <c r="H27" s="14" t="str">
+      <c r="H27" s="14">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1.0416666666642413</v>
       </c>
       <c r="I27" s="31"/>
       <c r="J27" s="31"/>
@@ -4379,12 +4387,12 @@
         <v>46302.041666666664</v>
       </c>
       <c r="F28" s="85">
-        <v>46302.166666666664</v>
+        <v>46302.125</v>
       </c>
       <c r="G28" s="14"/>
       <c r="H28" s="14">
         <f t="shared" si="0"/>
-        <v>1.125</v>
+        <v>1.0833333333357587</v>
       </c>
       <c r="I28" s="31"/>
       <c r="J28" s="31"/>
@@ -4446,23 +4454,20 @@
     <row r="29" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="45"/>
       <c r="B29" s="63" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C29" s="57" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D29" s="23"/>
       <c r="E29" s="85">
-        <v>46302.166666666664</v>
+        <v>46302.041666666664</v>
       </c>
       <c r="F29" s="85">
-        <v>46302.25</v>
+        <v>46302.208333333336</v>
       </c>
       <c r="G29" s="14"/>
-      <c r="H29" s="14">
-        <f t="shared" si="0"/>
-        <v>1.0833333333357587</v>
-      </c>
+      <c r="H29" s="14"/>
       <c r="I29" s="31"/>
       <c r="J29" s="31"/>
       <c r="K29" s="31"/>
@@ -4523,23 +4528,20 @@
     <row r="30" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="45"/>
       <c r="B30" s="63" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C30" s="57" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D30" s="23"/>
       <c r="E30" s="85">
-        <v>46302.25</v>
+        <v>46302.208333333336</v>
       </c>
       <c r="F30" s="85">
         <v>46302.291666666664</v>
       </c>
       <c r="G30" s="14"/>
-      <c r="H30" s="14">
-        <f t="shared" si="0"/>
-        <v>1.0416666666642413</v>
-      </c>
+      <c r="H30" s="14"/>
       <c r="I30" s="31"/>
       <c r="J30" s="31"/>
       <c r="K30" s="31"/>
@@ -4600,7 +4602,7 @@
     <row r="31" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="45"/>
       <c r="B31" s="63" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C31" s="57" t="s">
         <v>32</v>
@@ -4613,10 +4615,7 @@
         <v>46302.125</v>
       </c>
       <c r="G31" s="14"/>
-      <c r="H31" s="14">
-        <f t="shared" si="0"/>
-        <v>1.0833333333357587</v>
-      </c>
+      <c r="H31" s="14"/>
       <c r="I31" s="31"/>
       <c r="J31" s="31"/>
       <c r="K31" s="31"/>
@@ -4676,20 +4675,22 @@
     </row>
     <row r="32" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="45" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B32" s="63" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C32" s="57" t="s">
-        <v>32</v>
-      </c>
-      <c r="D32" s="23"/>
+        <v>20</v>
+      </c>
+      <c r="D32" s="23">
+        <v>0.8</v>
+      </c>
       <c r="E32" s="85">
-        <v>46302.041666666664</v>
+        <v>46303.125</v>
       </c>
       <c r="F32" s="85">
-        <v>46302.208333333336</v>
+        <v>46303.166666666664</v>
       </c>
       <c r="G32" s="14"/>
       <c r="H32" s="14"/>
@@ -4752,20 +4753,20 @@
     </row>
     <row r="33" spans="1:64" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A33" s="46" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B33" s="63" t="s">
         <v>50</v>
       </c>
       <c r="C33" s="57" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="D33" s="23"/>
       <c r="E33" s="85">
-        <v>46302.208333333336</v>
+        <v>46303.166666666664</v>
       </c>
       <c r="F33" s="85">
-        <v>46302.291666666664</v>
+        <v>46303.208333333336</v>
       </c>
       <c r="G33" s="14"/>
       <c r="H33" s="14"/>
@@ -4831,17 +4832,22 @@
         <v>51</v>
       </c>
       <c r="C34" s="57" t="s">
-        <v>32</v>
-      </c>
-      <c r="D34" s="23"/>
+        <v>20</v>
+      </c>
+      <c r="D34" s="23">
+        <v>0.5</v>
+      </c>
       <c r="E34" s="85">
-        <v>46302.041666666664</v>
+        <v>46303.208333333336</v>
       </c>
       <c r="F34" s="85">
-        <v>46302.125</v>
+        <v>46303.25</v>
       </c>
       <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
+      <c r="H34" s="14">
+        <f t="shared" si="0"/>
+        <v>1.0416666666642413</v>
+      </c>
       <c r="I34" s="31"/>
       <c r="J34" s="31"/>
       <c r="K34" s="31"/>
@@ -4900,21 +4906,18 @@
       <c r="BL34" s="31"/>
     </row>
     <row r="35" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="63" t="s">
+      <c r="B35" s="24" t="s">
         <v>52</v>
       </c>
-      <c r="C35" s="57" t="s">
-        <v>20</v>
-      </c>
-      <c r="D35" s="23"/>
-      <c r="E35" s="85">
-        <v>46303.125</v>
-      </c>
-      <c r="F35" s="85">
-        <v>46303.166666666664</v>
-      </c>
+      <c r="C35" s="58"/>
+      <c r="D35" s="25"/>
+      <c r="E35" s="75"/>
+      <c r="F35" s="76"/>
       <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
+      <c r="H35" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="I35" s="31"/>
       <c r="J35" s="31"/>
       <c r="K35" s="31"/>
@@ -4973,21 +4976,24 @@
       <c r="BL35" s="31"/>
     </row>
     <row r="36" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="63" t="s">
+      <c r="B36" s="64" t="s">
         <v>53</v>
       </c>
-      <c r="C36" s="57" t="s">
+      <c r="C36" s="59" t="s">
         <v>20</v>
       </c>
-      <c r="D36" s="23"/>
-      <c r="E36" s="85">
+      <c r="D36" s="26"/>
+      <c r="E36" s="86">
+        <v>46303.041666666664</v>
+      </c>
+      <c r="F36" s="86">
         <v>46303.166666666664</v>
       </c>
-      <c r="F36" s="85">
-        <v>46303.208333333336</v>
-      </c>
       <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
+      <c r="H36" s="14">
+        <f t="shared" si="0"/>
+        <v>1.125</v>
+      </c>
       <c r="I36" s="31"/>
       <c r="J36" s="31"/>
       <c r="K36" s="31"/>
@@ -5046,23 +5052,23 @@
       <c r="BL36" s="31"/>
     </row>
     <row r="37" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="63" t="s">
+      <c r="B37" s="64" t="s">
         <v>54</v>
       </c>
-      <c r="C37" s="57" t="s">
+      <c r="C37" s="59" t="s">
         <v>20</v>
       </c>
-      <c r="D37" s="23"/>
-      <c r="E37" s="85">
-        <v>46303.208333333336</v>
-      </c>
-      <c r="F37" s="85">
-        <v>46303.25</v>
+      <c r="D37" s="26"/>
+      <c r="E37" s="86">
+        <v>46303.166666666664</v>
+      </c>
+      <c r="F37" s="86">
+        <v>46303.291666666664</v>
       </c>
       <c r="G37" s="14"/>
       <c r="H37" s="14">
         <f t="shared" si="0"/>
-        <v>1.0416666666642413</v>
+        <v>1.125</v>
       </c>
       <c r="I37" s="31"/>
       <c r="J37" s="31"/>
@@ -5122,17 +5128,23 @@
       <c r="BL37" s="31"/>
     </row>
     <row r="38" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="24" t="s">
+      <c r="B38" s="64" t="s">
         <v>55</v>
       </c>
-      <c r="C38" s="58"/>
-      <c r="D38" s="25"/>
-      <c r="E38" s="75"/>
-      <c r="F38" s="76"/>
+      <c r="C38" s="59" t="s">
+        <v>20</v>
+      </c>
+      <c r="D38" s="26"/>
+      <c r="E38" s="86">
+        <v>46303.041666666664</v>
+      </c>
+      <c r="F38" s="86">
+        <v>46303.125</v>
+      </c>
       <c r="G38" s="14"/>
-      <c r="H38" s="14" t="str">
+      <c r="H38" s="14">
         <f t="shared" si="0"/>
-        <v/>
+        <v>1.0833333333357587</v>
       </c>
       <c r="I38" s="31"/>
       <c r="J38" s="31"/>
@@ -5196,7 +5208,7 @@
         <v>56</v>
       </c>
       <c r="C39" s="59" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D39" s="26"/>
       <c r="E39" s="86">
@@ -5272,7 +5284,7 @@
         <v>57</v>
       </c>
       <c r="C40" s="59" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D40" s="26"/>
       <c r="E40" s="86">
@@ -5344,24 +5356,21 @@
       <c r="BL40" s="31"/>
     </row>
     <row r="41" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="64" t="s">
+      <c r="B41" s="61" t="s">
         <v>58</v>
       </c>
-      <c r="C41" s="59" t="s">
-        <v>20</v>
-      </c>
-      <c r="D41" s="26"/>
-      <c r="E41" s="86">
+      <c r="C41" s="53" t="s">
+        <v>32</v>
+      </c>
+      <c r="D41" s="17"/>
+      <c r="E41" s="81">
         <v>46303.041666666664</v>
       </c>
-      <c r="F41" s="86">
+      <c r="F41" s="81">
         <v>46303.125</v>
       </c>
       <c r="G41" s="14"/>
-      <c r="H41" s="14">
-        <f t="shared" si="0"/>
-        <v>1.0833333333357587</v>
-      </c>
+      <c r="H41" s="14"/>
       <c r="I41" s="31"/>
       <c r="J41" s="31"/>
       <c r="K41" s="31"/>
@@ -5420,24 +5429,21 @@
       <c r="BL41" s="31"/>
     </row>
     <row r="42" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="64" t="s">
+      <c r="B42" s="61" t="s">
         <v>59</v>
       </c>
-      <c r="C42" s="59" t="s">
-        <v>32</v>
-      </c>
-      <c r="D42" s="26"/>
-      <c r="E42" s="86">
-        <v>46303.041666666664</v>
-      </c>
-      <c r="F42" s="86">
-        <v>46303.166666666664</v>
+      <c r="C42" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="D42" s="17"/>
+      <c r="E42" s="81">
+        <v>46304.041666666664</v>
+      </c>
+      <c r="F42" s="81">
+        <v>46304.166666666664</v>
       </c>
       <c r="G42" s="14"/>
-      <c r="H42" s="14">
-        <f t="shared" si="0"/>
-        <v>1.125</v>
-      </c>
+      <c r="H42" s="14"/>
       <c r="I42" s="31"/>
       <c r="J42" s="31"/>
       <c r="K42" s="31"/>
@@ -5496,24 +5502,21 @@
       <c r="BL42" s="31"/>
     </row>
     <row r="43" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="64" t="s">
+      <c r="B43" s="61" t="s">
         <v>60</v>
       </c>
-      <c r="C43" s="59" t="s">
-        <v>32</v>
-      </c>
-      <c r="D43" s="26"/>
-      <c r="E43" s="86">
-        <v>46303.166666666664</v>
-      </c>
-      <c r="F43" s="86">
-        <v>46303.291666666664</v>
+      <c r="C43" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="D43" s="17"/>
+      <c r="E43" s="81">
+        <v>46304.166666666664</v>
+      </c>
+      <c r="F43" s="81">
+        <v>46304.25</v>
       </c>
       <c r="G43" s="14"/>
-      <c r="H43" s="14">
-        <f t="shared" si="0"/>
-        <v>1.125</v>
-      </c>
+      <c r="H43" s="14"/>
       <c r="I43" s="31"/>
       <c r="J43" s="31"/>
       <c r="K43" s="31"/>
@@ -5576,14 +5579,14 @@
         <v>61</v>
       </c>
       <c r="C44" s="53" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="D44" s="17"/>
       <c r="E44" s="81">
-        <v>46303.041666666664</v>
+        <v>46304.25</v>
       </c>
       <c r="F44" s="81">
-        <v>46303.125</v>
+        <v>46304.291666666664</v>
       </c>
       <c r="G44" s="14"/>
       <c r="H44" s="14"/>
@@ -5649,7 +5652,7 @@
         <v>62</v>
       </c>
       <c r="C45" s="53" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D45" s="17"/>
       <c r="E45" s="81">
@@ -5722,14 +5725,14 @@
         <v>63</v>
       </c>
       <c r="C46" s="53" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D46" s="17"/>
       <c r="E46" s="81">
         <v>46304.166666666664</v>
       </c>
       <c r="F46" s="81">
-        <v>46304.25</v>
+        <v>46304.291666666664</v>
       </c>
       <c r="G46" s="14"/>
       <c r="H46" s="14"/>
@@ -5791,18 +5794,18 @@
       <c r="BL46" s="31"/>
     </row>
     <row r="47" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="61" t="s">
+      <c r="B47" s="64" t="s">
         <v>64</v>
       </c>
-      <c r="C47" s="53" t="s">
-        <v>20</v>
-      </c>
-      <c r="D47" s="17"/>
-      <c r="E47" s="81">
-        <v>46304.25</v>
-      </c>
-      <c r="F47" s="81">
-        <v>46304.291666666664</v>
+      <c r="C47" s="59" t="s">
+        <v>32</v>
+      </c>
+      <c r="D47" s="26"/>
+      <c r="E47" s="86">
+        <v>46304.041666666664</v>
+      </c>
+      <c r="F47" s="86">
+        <v>46304.125</v>
       </c>
       <c r="G47" s="14"/>
       <c r="H47" s="14"/>
@@ -5864,21 +5867,16 @@
       <c r="BL47" s="31"/>
     </row>
     <row r="48" spans="1:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="61" t="s">
-        <v>65</v>
-      </c>
-      <c r="C48" s="53" t="s">
-        <v>32</v>
-      </c>
-      <c r="D48" s="17"/>
-      <c r="E48" s="81">
-        <v>46304.041666666664</v>
-      </c>
-      <c r="F48" s="81">
-        <v>46304.166666666664</v>
-      </c>
+      <c r="B48" s="65"/>
+      <c r="C48" s="60"/>
+      <c r="D48" s="13"/>
+      <c r="E48" s="77"/>
+      <c r="F48" s="77"/>
       <c r="G48" s="14"/>
-      <c r="H48" s="14"/>
+      <c r="H48" s="14" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
       <c r="I48" s="31"/>
       <c r="J48" s="31"/>
       <c r="K48" s="31"/>
@@ -5937,298 +5935,84 @@
       <c r="BL48" s="31"/>
     </row>
     <row r="49" spans="2:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="61" t="s">
-        <v>66</v>
-      </c>
-      <c r="C49" s="53" t="s">
-        <v>32</v>
-      </c>
-      <c r="D49" s="17"/>
-      <c r="E49" s="81">
-        <v>46304.166666666664</v>
-      </c>
-      <c r="F49" s="81">
-        <v>46304.291666666664</v>
-      </c>
-      <c r="G49" s="14"/>
-      <c r="H49" s="14"/>
-      <c r="I49" s="31"/>
-      <c r="J49" s="31"/>
-      <c r="K49" s="31"/>
-      <c r="L49" s="31"/>
-      <c r="M49" s="31"/>
-      <c r="N49" s="31"/>
-      <c r="O49" s="31"/>
-      <c r="P49" s="31"/>
-      <c r="Q49" s="31"/>
-      <c r="R49" s="31"/>
-      <c r="S49" s="31"/>
-      <c r="T49" s="31"/>
-      <c r="U49" s="31"/>
-      <c r="V49" s="31"/>
-      <c r="W49" s="31"/>
-      <c r="X49" s="31"/>
-      <c r="Y49" s="31"/>
-      <c r="Z49" s="31"/>
-      <c r="AA49" s="31"/>
-      <c r="AB49" s="31"/>
-      <c r="AC49" s="31"/>
-      <c r="AD49" s="31"/>
-      <c r="AE49" s="31"/>
-      <c r="AF49" s="31"/>
-      <c r="AG49" s="31"/>
-      <c r="AH49" s="31"/>
-      <c r="AI49" s="31"/>
-      <c r="AJ49" s="31"/>
-      <c r="AK49" s="31"/>
-      <c r="AL49" s="31"/>
-      <c r="AM49" s="31"/>
-      <c r="AN49" s="31"/>
-      <c r="AO49" s="31"/>
-      <c r="AP49" s="31"/>
-      <c r="AQ49" s="31"/>
-      <c r="AR49" s="31"/>
-      <c r="AS49" s="31"/>
-      <c r="AT49" s="31"/>
-      <c r="AU49" s="31"/>
-      <c r="AV49" s="31"/>
-      <c r="AW49" s="31"/>
-      <c r="AX49" s="31"/>
-      <c r="AY49" s="31"/>
-      <c r="AZ49" s="31"/>
-      <c r="BA49" s="31"/>
-      <c r="BB49" s="31"/>
-      <c r="BC49" s="31"/>
-      <c r="BD49" s="31"/>
-      <c r="BE49" s="31"/>
-      <c r="BF49" s="31"/>
-      <c r="BG49" s="31"/>
-      <c r="BH49" s="31"/>
-      <c r="BI49" s="31"/>
-      <c r="BJ49" s="31"/>
-      <c r="BK49" s="31"/>
-      <c r="BL49" s="31"/>
-    </row>
-    <row r="50" spans="2:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B50" s="64" t="s">
-        <v>67</v>
-      </c>
-      <c r="C50" s="59" t="s">
-        <v>32</v>
-      </c>
-      <c r="D50" s="26"/>
-      <c r="E50" s="86">
-        <v>46304.041666666664</v>
-      </c>
-      <c r="F50" s="86">
-        <v>46304.125</v>
-      </c>
-      <c r="G50" s="14"/>
-      <c r="H50" s="14"/>
-      <c r="I50" s="31"/>
-      <c r="J50" s="31"/>
-      <c r="K50" s="31"/>
-      <c r="L50" s="31"/>
-      <c r="M50" s="31"/>
-      <c r="N50" s="31"/>
-      <c r="O50" s="31"/>
-      <c r="P50" s="31"/>
-      <c r="Q50" s="31"/>
-      <c r="R50" s="31"/>
-      <c r="S50" s="31"/>
-      <c r="T50" s="31"/>
-      <c r="U50" s="31"/>
-      <c r="V50" s="31"/>
-      <c r="W50" s="31"/>
-      <c r="X50" s="31"/>
-      <c r="Y50" s="31"/>
-      <c r="Z50" s="31"/>
-      <c r="AA50" s="31"/>
-      <c r="AB50" s="31"/>
-      <c r="AC50" s="31"/>
-      <c r="AD50" s="31"/>
-      <c r="AE50" s="31"/>
-      <c r="AF50" s="31"/>
-      <c r="AG50" s="31"/>
-      <c r="AH50" s="31"/>
-      <c r="AI50" s="31"/>
-      <c r="AJ50" s="31"/>
-      <c r="AK50" s="31"/>
-      <c r="AL50" s="31"/>
-      <c r="AM50" s="31"/>
-      <c r="AN50" s="31"/>
-      <c r="AO50" s="31"/>
-      <c r="AP50" s="31"/>
-      <c r="AQ50" s="31"/>
-      <c r="AR50" s="31"/>
-      <c r="AS50" s="31"/>
-      <c r="AT50" s="31"/>
-      <c r="AU50" s="31"/>
-      <c r="AV50" s="31"/>
-      <c r="AW50" s="31"/>
-      <c r="AX50" s="31"/>
-      <c r="AY50" s="31"/>
-      <c r="AZ50" s="31"/>
-      <c r="BA50" s="31"/>
-      <c r="BB50" s="31"/>
-      <c r="BC50" s="31"/>
-      <c r="BD50" s="31"/>
-      <c r="BE50" s="31"/>
-      <c r="BF50" s="31"/>
-      <c r="BG50" s="31"/>
-      <c r="BH50" s="31"/>
-      <c r="BI50" s="31"/>
-      <c r="BJ50" s="31"/>
-      <c r="BK50" s="31"/>
-      <c r="BL50" s="31"/>
-    </row>
-    <row r="51" spans="2:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B51" s="65"/>
-      <c r="C51" s="60"/>
-      <c r="D51" s="13"/>
-      <c r="E51" s="77"/>
-      <c r="F51" s="77"/>
-      <c r="G51" s="14"/>
-      <c r="H51" s="14" t="str">
+      <c r="B49" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="C49" s="28"/>
+      <c r="D49" s="29"/>
+      <c r="E49" s="78"/>
+      <c r="F49" s="79"/>
+      <c r="G49" s="30"/>
+      <c r="H49" s="30" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="I51" s="31"/>
-      <c r="J51" s="31"/>
-      <c r="K51" s="31"/>
-      <c r="L51" s="31"/>
-      <c r="M51" s="31"/>
-      <c r="N51" s="31"/>
-      <c r="O51" s="31"/>
-      <c r="P51" s="31"/>
-      <c r="Q51" s="31"/>
-      <c r="R51" s="31"/>
-      <c r="S51" s="31"/>
-      <c r="T51" s="31"/>
-      <c r="U51" s="31"/>
-      <c r="V51" s="31"/>
-      <c r="W51" s="31"/>
-      <c r="X51" s="31"/>
-      <c r="Y51" s="31"/>
-      <c r="Z51" s="31"/>
-      <c r="AA51" s="31"/>
-      <c r="AB51" s="31"/>
-      <c r="AC51" s="31"/>
-      <c r="AD51" s="31"/>
-      <c r="AE51" s="31"/>
-      <c r="AF51" s="31"/>
-      <c r="AG51" s="31"/>
-      <c r="AH51" s="31"/>
-      <c r="AI51" s="31"/>
-      <c r="AJ51" s="31"/>
-      <c r="AK51" s="31"/>
-      <c r="AL51" s="31"/>
-      <c r="AM51" s="31"/>
-      <c r="AN51" s="31"/>
-      <c r="AO51" s="31"/>
-      <c r="AP51" s="31"/>
-      <c r="AQ51" s="31"/>
-      <c r="AR51" s="31"/>
-      <c r="AS51" s="31"/>
-      <c r="AT51" s="31"/>
-      <c r="AU51" s="31"/>
-      <c r="AV51" s="31"/>
-      <c r="AW51" s="31"/>
-      <c r="AX51" s="31"/>
-      <c r="AY51" s="31"/>
-      <c r="AZ51" s="31"/>
-      <c r="BA51" s="31"/>
-      <c r="BB51" s="31"/>
-      <c r="BC51" s="31"/>
-      <c r="BD51" s="31"/>
-      <c r="BE51" s="31"/>
-      <c r="BF51" s="31"/>
-      <c r="BG51" s="31"/>
-      <c r="BH51" s="31"/>
-      <c r="BI51" s="31"/>
-      <c r="BJ51" s="31"/>
-      <c r="BK51" s="31"/>
-      <c r="BL51" s="31"/>
-    </row>
-    <row r="52" spans="2:64" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="27" t="s">
-        <v>68</v>
-      </c>
-      <c r="C52" s="28"/>
-      <c r="D52" s="29"/>
-      <c r="E52" s="78"/>
-      <c r="F52" s="79"/>
-      <c r="G52" s="30"/>
-      <c r="H52" s="30" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="I52" s="33"/>
-      <c r="J52" s="33"/>
-      <c r="K52" s="33"/>
-      <c r="L52" s="33"/>
-      <c r="M52" s="33"/>
-      <c r="N52" s="33"/>
-      <c r="O52" s="33"/>
-      <c r="P52" s="33"/>
-      <c r="Q52" s="33"/>
-      <c r="R52" s="33"/>
-      <c r="S52" s="33"/>
-      <c r="T52" s="33"/>
-      <c r="U52" s="33"/>
-      <c r="V52" s="33"/>
-      <c r="W52" s="33"/>
-      <c r="X52" s="33"/>
-      <c r="Y52" s="33"/>
-      <c r="Z52" s="33"/>
-      <c r="AA52" s="33"/>
-      <c r="AB52" s="33"/>
-      <c r="AC52" s="33"/>
-      <c r="AD52" s="33"/>
-      <c r="AE52" s="33"/>
-      <c r="AF52" s="33"/>
-      <c r="AG52" s="33"/>
-      <c r="AH52" s="33"/>
-      <c r="AI52" s="33"/>
-      <c r="AJ52" s="33"/>
-      <c r="AK52" s="33"/>
-      <c r="AL52" s="33"/>
-      <c r="AM52" s="33"/>
-      <c r="AN52" s="33"/>
-      <c r="AO52" s="33"/>
-      <c r="AP52" s="33"/>
-      <c r="AQ52" s="33"/>
-      <c r="AR52" s="33"/>
-      <c r="AS52" s="33"/>
-      <c r="AT52" s="33"/>
-      <c r="AU52" s="33"/>
-      <c r="AV52" s="33"/>
-      <c r="AW52" s="33"/>
-      <c r="AX52" s="33"/>
-      <c r="AY52" s="33"/>
-      <c r="AZ52" s="33"/>
-      <c r="BA52" s="33"/>
-      <c r="BB52" s="33"/>
-      <c r="BC52" s="33"/>
-      <c r="BD52" s="33"/>
-      <c r="BE52" s="33"/>
-      <c r="BF52" s="33"/>
-      <c r="BG52" s="33"/>
-      <c r="BH52" s="33"/>
-      <c r="BI52" s="33"/>
-      <c r="BJ52" s="33"/>
-      <c r="BK52" s="33"/>
-      <c r="BL52" s="33"/>
-    </row>
-    <row r="53" spans="2:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="G53" s="6"/>
-    </row>
-    <row r="54" spans="2:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C54" s="11"/>
-      <c r="F54" s="47"/>
-    </row>
-    <row r="55" spans="2:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C55" s="12"/>
+      <c r="I49" s="33"/>
+      <c r="J49" s="33"/>
+      <c r="K49" s="33"/>
+      <c r="L49" s="33"/>
+      <c r="M49" s="33"/>
+      <c r="N49" s="33"/>
+      <c r="O49" s="33"/>
+      <c r="P49" s="33"/>
+      <c r="Q49" s="33"/>
+      <c r="R49" s="33"/>
+      <c r="S49" s="33"/>
+      <c r="T49" s="33"/>
+      <c r="U49" s="33"/>
+      <c r="V49" s="33"/>
+      <c r="W49" s="33"/>
+      <c r="X49" s="33"/>
+      <c r="Y49" s="33"/>
+      <c r="Z49" s="33"/>
+      <c r="AA49" s="33"/>
+      <c r="AB49" s="33"/>
+      <c r="AC49" s="33"/>
+      <c r="AD49" s="33"/>
+      <c r="AE49" s="33"/>
+      <c r="AF49" s="33"/>
+      <c r="AG49" s="33"/>
+      <c r="AH49" s="33"/>
+      <c r="AI49" s="33"/>
+      <c r="AJ49" s="33"/>
+      <c r="AK49" s="33"/>
+      <c r="AL49" s="33"/>
+      <c r="AM49" s="33"/>
+      <c r="AN49" s="33"/>
+      <c r="AO49" s="33"/>
+      <c r="AP49" s="33"/>
+      <c r="AQ49" s="33"/>
+      <c r="AR49" s="33"/>
+      <c r="AS49" s="33"/>
+      <c r="AT49" s="33"/>
+      <c r="AU49" s="33"/>
+      <c r="AV49" s="33"/>
+      <c r="AW49" s="33"/>
+      <c r="AX49" s="33"/>
+      <c r="AY49" s="33"/>
+      <c r="AZ49" s="33"/>
+      <c r="BA49" s="33"/>
+      <c r="BB49" s="33"/>
+      <c r="BC49" s="33"/>
+      <c r="BD49" s="33"/>
+      <c r="BE49" s="33"/>
+      <c r="BF49" s="33"/>
+      <c r="BG49" s="33"/>
+      <c r="BH49" s="33"/>
+      <c r="BI49" s="33"/>
+      <c r="BJ49" s="33"/>
+      <c r="BK49" s="33"/>
+      <c r="BL49" s="33"/>
+    </row>
+    <row r="50" spans="2:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="G50" s="6"/>
+    </row>
+    <row r="51" spans="2:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C51" s="11"/>
+      <c r="F51" s="47"/>
+    </row>
+    <row r="52" spans="2:64" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C52" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="11">
@@ -6244,7 +6028,7 @@
     <mergeCell ref="AR4:AX4"/>
     <mergeCell ref="AY4:BE4"/>
   </mergeCells>
-  <conditionalFormatting sqref="D7:D52">
+  <conditionalFormatting sqref="D7:D49">
     <cfRule type="dataBar" priority="18">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -6258,13 +6042,13 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:BL52">
-    <cfRule type="expression" dxfId="3" priority="37">
+  <conditionalFormatting sqref="I5:BL49">
+    <cfRule type="expression" dxfId="2" priority="37">
       <formula>AND(TODAY()&gt;=I$5,TODAY()&lt;J$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I7:BL52">
-    <cfRule type="expression" dxfId="2" priority="32">
+  <conditionalFormatting sqref="I7:BL49">
+    <cfRule type="expression" dxfId="1" priority="32">
       <formula>AND(task_end&gt;=I$5,task_start&lt;J$5)</formula>
     </cfRule>
   </conditionalFormatting>
@@ -6295,7 +6079,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D7:D52</xm:sqref>
+          <xm:sqref>D7:D49</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -6320,31 +6104,31 @@
   <sheetData>
     <row r="1" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A1" s="87" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" s="87" t="s">
+        <v>67</v>
+      </c>
+      <c r="C1" s="87" t="s">
+        <v>68</v>
+      </c>
+      <c r="D1" s="87" t="s">
         <v>69</v>
       </c>
-      <c r="B1" s="87" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1" s="87" t="s">
-        <v>71</v>
-      </c>
-      <c r="D1" s="87" t="s">
-        <v>72</v>
-      </c>
       <c r="E1" s="87" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="F1" s="87" t="s">
+        <v>177</v>
+      </c>
+      <c r="G1" s="87" t="s">
+        <v>178</v>
+      </c>
+      <c r="H1" s="100" t="s">
+        <v>152</v>
+      </c>
+      <c r="I1" s="87" t="s">
         <v>180</v>
-      </c>
-      <c r="G1" s="87" t="s">
-        <v>181</v>
-      </c>
-      <c r="H1" s="100" t="s">
-        <v>155</v>
-      </c>
-      <c r="I1" s="87" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="45" x14ac:dyDescent="0.25">
@@ -6352,13 +6136,13 @@
         <v>19</v>
       </c>
       <c r="B2" s="88" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C2" s="88" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D2" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E2">
         <v>5</v>
@@ -6380,16 +6164,16 @@
     </row>
     <row r="3" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="87" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="88" t="s">
+        <v>74</v>
+      </c>
+      <c r="C3" s="88" t="s">
+        <v>75</v>
+      </c>
+      <c r="D3" s="99" t="s">
         <v>76</v>
-      </c>
-      <c r="B3" s="88" t="s">
-        <v>77</v>
-      </c>
-      <c r="C3" s="88" t="s">
-        <v>78</v>
-      </c>
-      <c r="D3" s="99" t="s">
-        <v>79</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -6411,16 +6195,16 @@
     </row>
     <row r="4" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="87" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B4" s="88" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="C4" s="88" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D4" s="99" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E4">
         <v>3</v>
@@ -6445,13 +6229,13 @@
         <v>22</v>
       </c>
       <c r="B5" s="88" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="C5" s="88" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="D5" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E5">
         <v>4</v>
@@ -6473,16 +6257,16 @@
     </row>
     <row r="6" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A6" s="87" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B6" s="88" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C6" s="88" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D6" s="99" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E6">
         <v>3</v>
@@ -6504,16 +6288,16 @@
     </row>
     <row r="7" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A7" s="87" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B7" s="88" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="C7" s="88" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="D7" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E7">
         <v>5</v>
@@ -6535,16 +6319,16 @@
     </row>
     <row r="8" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A8" s="87" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B8" s="88" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C8" s="88" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="D8" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E8">
         <v>5</v>
@@ -6566,16 +6350,16 @@
     </row>
     <row r="9" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A9" s="87" t="s">
+        <v>89</v>
+      </c>
+      <c r="B9" s="88" t="s">
+        <v>90</v>
+      </c>
+      <c r="C9" s="88" t="s">
+        <v>91</v>
+      </c>
+      <c r="D9" s="99" t="s">
         <v>92</v>
-      </c>
-      <c r="B9" s="88" t="s">
-        <v>93</v>
-      </c>
-      <c r="C9" s="88" t="s">
-        <v>94</v>
-      </c>
-      <c r="D9" s="99" t="s">
-        <v>95</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -6597,16 +6381,16 @@
     </row>
     <row r="10" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" s="87" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B10" s="88" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C10" s="88" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D10" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E10">
         <v>5</v>
@@ -6628,16 +6412,16 @@
     </row>
     <row r="11" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A11" s="87" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B11" s="102" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C11" s="88" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D11" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E11">
         <v>4</v>
@@ -6659,16 +6443,16 @@
     </row>
     <row r="12" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A12" s="87" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B12" s="88" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C12" s="88" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="D12" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E12">
         <v>5</v>
@@ -6690,16 +6474,16 @@
     </row>
     <row r="13" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A13" s="87" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B13" s="88" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C13" s="88" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="D13" s="99" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E13">
         <v>3</v>
@@ -6721,16 +6505,16 @@
     </row>
     <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="87" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B14" s="88" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C14" s="88" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="D14" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E14">
         <v>4</v>
@@ -6752,16 +6536,16 @@
     </row>
     <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="87" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B15" s="88" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C15" s="88" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D15" s="99" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E15">
         <v>3</v>
@@ -6783,16 +6567,16 @@
     </row>
     <row r="16" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A16" s="87" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B16" s="88" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C16" s="88" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="D16" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E16">
         <v>4</v>
@@ -6814,16 +6598,16 @@
     </row>
     <row r="17" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A17" s="87" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B17" s="88" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C17" s="88" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="D17" s="99" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E17">
         <v>3</v>
@@ -6845,16 +6629,16 @@
     </row>
     <row r="18" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A18" s="87" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B18" s="88" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C18" s="88" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="D18" s="99" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E18">
         <v>2</v>
@@ -6876,16 +6660,16 @@
     </row>
     <row r="19" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A19" s="87" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B19" s="88" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C19" s="88" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D19" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E19">
         <v>5</v>
@@ -6907,16 +6691,16 @@
     </row>
     <row r="20" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="87" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B20" s="88" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C20" s="88" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="D20" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E20">
         <v>4</v>
@@ -6938,16 +6722,16 @@
     </row>
     <row r="21" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="87" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B21" s="88" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C21" s="88" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="D21" s="99" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="E21">
         <v>2</v>
@@ -6969,16 +6753,16 @@
     </row>
     <row r="22" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="87" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="B22" s="88" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C22" s="88" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D22" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E22">
         <v>4</v>
@@ -7000,16 +6784,16 @@
     </row>
     <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="87" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B23" s="88" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C23" s="88" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="D23" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E23">
         <v>4</v>
@@ -7031,16 +6815,16 @@
     </row>
     <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="87" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B24" s="88" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C24" s="88" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="D24" s="99" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E24">
         <v>4</v>
@@ -7062,16 +6846,16 @@
     </row>
     <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="87" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B25" s="88" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C25" s="88" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="D25" s="99" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E25">
         <v>5</v>
@@ -7093,16 +6877,16 @@
     </row>
     <row r="26" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A26" s="87" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B26" s="88" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="C26" s="88" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="D26" s="99" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E26">
         <v>3</v>
@@ -7124,16 +6908,16 @@
     </row>
     <row r="27" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A27" s="87" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="B27" s="88" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="C27" s="88" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D27" s="99" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E27">
         <v>3</v>
@@ -7155,7 +6939,7 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D28" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="E28">
         <f>SUM(E2:E27)*5</f>
@@ -7172,7 +6956,7 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="D29" s="99" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E29" s="101">
         <f>_xlfn.PERCENTOF(E28,E28)</f>
@@ -7189,16 +6973,16 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="91" t="s">
+        <v>145</v>
+      </c>
+      <c r="B31" s="91" t="s">
+        <v>146</v>
+      </c>
+      <c r="C31" s="91" t="s">
+        <v>147</v>
+      </c>
+      <c r="D31" s="92" t="s">
         <v>148</v>
-      </c>
-      <c r="B31" s="91" t="s">
-        <v>149</v>
-      </c>
-      <c r="C31" s="91" t="s">
-        <v>150</v>
-      </c>
-      <c r="D31" s="92" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
@@ -7206,13 +6990,13 @@
         <v>1</v>
       </c>
       <c r="B32" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C32" s="89" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D32" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
@@ -7220,13 +7004,13 @@
         <v>2</v>
       </c>
       <c r="B33" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C33" s="89" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="D33" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -7234,13 +7018,13 @@
         <v>3</v>
       </c>
       <c r="B34" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="C34" s="90" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D34" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -7248,33 +7032,33 @@
         <v>4</v>
       </c>
       <c r="B35" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C35" s="89" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="D35" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B37" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B38" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B39" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A2:I27">
-    <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="Hoch">
+    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Hoch">
       <formula>NOT(ISERROR(SEARCH("Hoch",A2)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7300,79 +7084,79 @@
     <row r="1" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="2" spans="1:2" s="37" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="36" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="B2" s="36"/>
     </row>
     <row r="3" spans="1:2" s="41" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="68" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="B3" s="42"/>
     </row>
     <row r="4" spans="1:2" s="38" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A4" s="39" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="74.099999999999994" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="40" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="39" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" spans="1:2" s="35" customFormat="1" ht="204.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="44" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="8" spans="1:2" s="38" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A8" s="39" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="75" x14ac:dyDescent="0.2">
       <c r="A9" s="40" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="10" spans="1:2" s="35" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="43" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="11" spans="1:2" s="38" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A11" s="39" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="12" spans="1:2" ht="45" x14ac:dyDescent="0.2">
       <c r="A12" s="40" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="1:2" s="35" customFormat="1" ht="27.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="43" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="14" spans="1:2" s="38" customFormat="1" ht="26.25" x14ac:dyDescent="0.4">
       <c r="A14" s="39" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="40" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="90" x14ac:dyDescent="0.2">
       <c r="A16" s="40" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
   </sheetData>

</xml_diff>